<commit_message>
fix(ghost): clear SharePoint schema IDs from Office custom XML properties
Testing with real Microsoft Office files showed customXml/itemPropsN.xml
was copied unchanged. SharePoint lists its own schemas there by GUIDs that
identify the site, and the same GUIDs appeared in two unrelated files, so
stripped documents could still be linked to one organisation. Replace each
itemProps part with an empty one (neutral, per-package item ID), and drop
Word content-control data bindings, which name the same store and
namespaces; bound controls keep their current text.

Fixtures now plant the sentinel in an itemProps part and a dataBinding.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WcDieTZkDaYco9mAoob18S
</commit_message>
<xml_diff>
--- a/tests/js/fixtures/sample.xlsx
+++ b/tests/js/fixtures/sample.xlsx
@@ -104,4 +104,13 @@
     <DisplayName>ZQX7731</DisplayName>
   </Owner>
 </p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ZQX7731-0000-0000-0000-000000000001}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="ZQX7731-6b5d-4628-b7e0-5b86efa98958"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>